<commit_message>
add image to localStorage, fix disable button
</commit_message>
<xml_diff>
--- a/public/files/template_soal.xlsx
+++ b/public/files/template_soal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FC144BC9-0DC2-4055-8130-AD6966498362}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8E634F6-F60E-460D-947C-0251D3240E8F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B37F4553-3839-4BC5-BB58-27AE0A685357}"/>
+    <workbookView xWindow="4710" yWindow="4335" windowWidth="25500" windowHeight="11295" xr2:uid="{B37F4553-3839-4BC5-BB58-27AE0A685357}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
   <si>
     <t>pertanyaan</t>
   </si>
@@ -64,6 +64,12 @@
   </si>
   <si>
     <t>d</t>
+  </si>
+  <si>
+    <t>gambar</t>
+  </si>
+  <si>
+    <t>isikan nama file soal</t>
   </si>
 </sst>
 </file>
@@ -429,10 +435,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E52F5882-2780-41F7-B99D-85D1964CE165}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -451,8 +457,11 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -471,8 +480,11 @@
       <c r="F2" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="G2" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>

</xml_diff>